<commit_message>
feat(naming): 为polarisKitexInstance添加Tags方法获取所有标签 refactor(resolver): 移除Resolver接口，直接使用discovery.Resolver refactor(mysql): 重构mysql初始化逻辑，使用服务发现获取配置 feat(nano): 在NanoInitService中添加服务注册与注销功能 chore: 更新依赖版本
</commit_message>
<xml_diff>
--- a/servers/maze_main_server_dev/conf.d/data/git_version_v8【配表版本号】.xlsx
+++ b/servers/maze_main_server_dev/conf.d/data/git_version_v8【配表版本号】.xlsx
@@ -486,12 +486,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9631cd168025762c1c7487f0b95be890f47c1887</t>
+          <t>10842e4073bbf3623f52f2788a0880140ef1d9f5</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-06-10 12:04:30</t>
+          <t>2025-06-13 17:17:02</t>
         </is>
       </c>
     </row>

</xml_diff>